<commit_message>
Leakage nach dem Locked-Box-Stichtag
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WS5ibq7ARdN5REenEkuqwT
</commit_message>
<xml_diff>
--- a/beispiele/gross/datenraum/12.1 Q&A-Liste Projekt Säntis.xlsx
+++ b/beispiele/gross/datenraum/12.1 Q&A-Liste Projekt Säntis.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,6 +516,26 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>19.08.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Gab es seit dem 31.12.2025 Zahlungen an die Aktionärin?</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Am 15.03.2026 wurde eine Management Fee von CHF 60'000 an die Rohner Holding AG bezahlt.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>26.08.2026</t>
         </is>
       </c>
     </row>

</xml_diff>